<commit_message>
commit "third push of project"
</commit_message>
<xml_diff>
--- a/VtigerCRMHybridFramework/src/test/resources/Test_Data/VtigerTestData.xlsx
+++ b/VtigerCRMHybridFramework/src/test/resources/Test_Data/VtigerTestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{6FF4739D-DAA9-4DDF-A513-BE70B65DE044}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{3952E3B4-E06B-4AE1-8BB6-D9778F87C82F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="5" xr2:uid="{30AABFC3-966B-4924-A5F9-1D41A7EB3098}"/>
   </bookViews>
@@ -18,7 +18,7 @@
     <sheet name="Sheet8" sheetId="11" r:id="rId8"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1"/>
+  <oleSize ref="A1:L9"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="59">
   <si>
     <t>title</t>
   </si>
@@ -180,9 +180,6 @@
     <t>emailName</t>
   </si>
   <si>
-    <t>Vinayak Malgaund</t>
-  </si>
-  <si>
     <t>SubjectName</t>
   </si>
   <si>
@@ -216,7 +213,7 @@
     <t>Application issue handle</t>
   </si>
   <si>
-    <t>Acceptance Proposal</t>
+    <t>kushi rajkumari</t>
   </si>
 </sst>
 </file>
@@ -610,7 +607,7 @@
         <v>10</v>
       </c>
       <c r="E1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -627,7 +624,7 @@
         <v>11</v>
       </c>
       <c r="E2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -895,23 +892,23 @@
         <v>46</v>
       </c>
       <c r="B1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -930,26 +927,26 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" t="s">
         <v>51</v>
-      </c>
-      <c r="B1" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -972,23 +969,23 @@
         <v>46</v>
       </c>
       <c r="B1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>